<commit_message>
Docs: update diagram and data dictionary
Diagram: add shop_10 box, scraper is now weekly on Mac with Claude
extraction, retry is up to 4 retries with backoff, version date
2026/10/28. Data dictionary spreadsheet updated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Documentation/Statement_Data_Dictionary_Naming_Conventions_&_Lookup Tables.xlsx
+++ b/03_Documentation/Statement_Data_Dictionary_Naming_Conventions_&_Lookup Tables.xlsx
@@ -507,7 +507,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Data dictionary, naming conventions and lookup tables. Version V2, 2026-10-24. Project statement-competitor-pipeline, dataset statement_competitor_data_warehouse (Google BigQuery).</t>
+          <t>Data dictionary, naming conventions and lookup tables. Version V2, 2026-10-24 (updated 2026-10-28). Project statement-competitor-pipeline, dataset statement_competitor_data_warehouse (Google BigQuery).</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Manual (seeded by 01_DDL/04)</t>
+          <t>Manual (seeded by 01_DDL/04a)</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Manual (default row seeded by 01_DDL/04)</t>
+          <t>Manual (default row seeded by 01_DDL/04, shop exceptions by 04a)</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>What the scraper delivers to the Cloud Storage bucket. Upload the run summary first, then the products CSV. Use dated names, e.g. MCM_All_products_20261027.csv.</t>
+          <t>What the scraper delivers to the Cloud Storage bucket. Upload the run summary first, then the products CSV. Use dated names, e.g. MCM_All_products_2026-10-27.csv.</t>
         </is>
       </c>
     </row>
@@ -11703,7 +11703,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Verified coordinates per shop. Overrides scraped coordinates in step 4. Matched case-insensitively. Values are seeded in 01_DDL/04_create_reference_tables.sql; add new shops there or with an INSERT.</t>
+          <t>Verified coordinates per shop. Overrides scraped coordinates in step 4. Matched case-insensitively. Values are seeded by 01_DDL/04a_seed_shops.sql (local only; 04a_seed_shops.example.sql shows the format); add new shops there or with an INSERT.</t>
         </is>
       </c>
     </row>
@@ -14580,12 +14580,12 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>&lt;name&gt;_&lt;YYYYMMDD&gt;.csv</t>
+          <t>&lt;name&gt;_&lt;YYYY-MM-DD&gt;.csv</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>MCM_All_products_20261027.csv</t>
+          <t>MCM_All_products_2026-10-27.csv</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -14607,7 +14607,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>MCM_All_products_20261027_run_summary.csv</t>
+          <t>MCM_All_products_2026-10-27_run_summary.csv</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">

</xml_diff>